<commit_message>
added data to seminole
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Seminole/Seminole Freedman Two.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Seminole/Seminole Freedman Two.xlsx
@@ -390,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -440,6 +440,779 @@
         <v>14</v>
       </c>
     </row>
+    <row r="2" spans="1:15">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3">
+        <f>A2+1</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4">
+        <f t="shared" ref="A4:A67" si="0">A3+1</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68">
+        <f t="shared" ref="A68:A130" si="1">A67+1</f>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69">
+        <f t="shared" si="1"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71">
+        <f t="shared" si="1"/>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72">
+        <f t="shared" si="1"/>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73">
+        <f t="shared" si="1"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74">
+        <f t="shared" si="1"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75">
+        <f t="shared" si="1"/>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77">
+        <f t="shared" si="1"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78">
+        <f t="shared" si="1"/>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79">
+        <f t="shared" si="1"/>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80">
+        <f t="shared" si="1"/>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82">
+        <f t="shared" si="1"/>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83">
+        <f t="shared" si="1"/>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84">
+        <f t="shared" si="1"/>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85">
+        <f t="shared" si="1"/>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86">
+        <f t="shared" si="1"/>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87">
+        <f t="shared" si="1"/>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88">
+        <f t="shared" si="1"/>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89">
+        <f t="shared" si="1"/>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90">
+        <f t="shared" si="1"/>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92">
+        <f t="shared" si="1"/>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93">
+        <f t="shared" si="1"/>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94">
+        <f t="shared" si="1"/>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95">
+        <f t="shared" si="1"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96">
+        <f t="shared" si="1"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97">
+        <f t="shared" si="1"/>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98">
+        <f t="shared" si="1"/>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99">
+        <f t="shared" si="1"/>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100">
+        <f t="shared" si="1"/>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102">
+        <f t="shared" si="1"/>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103">
+        <f t="shared" si="1"/>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104">
+        <f t="shared" si="1"/>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105">
+        <f t="shared" si="1"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106">
+        <f t="shared" si="1"/>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107">
+        <f t="shared" si="1"/>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108">
+        <f t="shared" si="1"/>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109">
+        <f t="shared" si="1"/>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110">
+        <f t="shared" si="1"/>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111">
+        <f t="shared" si="1"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112">
+        <f t="shared" si="1"/>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113">
+        <f t="shared" si="1"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114">
+        <f t="shared" si="1"/>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115">
+        <f t="shared" si="1"/>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116">
+        <f t="shared" si="1"/>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117">
+        <f t="shared" si="1"/>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118">
+        <f t="shared" si="1"/>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119">
+        <f t="shared" si="1"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120">
+        <f t="shared" si="1"/>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122">
+        <f t="shared" si="1"/>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123">
+        <f t="shared" si="1"/>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124">
+        <f t="shared" si="1"/>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125">
+        <f t="shared" si="1"/>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126">
+        <f t="shared" si="1"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128">
+        <f t="shared" si="1"/>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129">
+        <f t="shared" si="1"/>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130">
+        <f t="shared" si="1"/>
+        <v>129</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added data to seminole freedman
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Seminole/Seminole Freedman Two.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Seminole/Seminole Freedman Two.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -65,6 +65,12 @@
   </si>
   <si>
     <t>Freedman</t>
+  </si>
+  <si>
+    <t>Dawes Rolls Full Document - Creek By Blood - Page 633</t>
+  </si>
+  <si>
+    <t>Dawes Rolls Full Document - Creek By Blood - Page 634</t>
   </si>
 </sst>
 </file>
@@ -401,6 +407,7 @@
   <cols>
     <col min="2" max="2" width="11.5703125" customWidth="1"/>
     <col min="12" max="12" width="14.5703125" customWidth="1"/>
+    <col min="14" max="14" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -457,8 +464,14 @@
       <c r="B2" t="s">
         <v>15</v>
       </c>
+      <c r="C2">
+        <v>633</v>
+      </c>
       <c r="L2" t="s">
         <v>16</v>
+      </c>
+      <c r="N2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -469,8 +482,16 @@
       <c r="B3" t="s">
         <v>15</v>
       </c>
+      <c r="C3">
+        <f>C2</f>
+        <v>633</v>
+      </c>
       <c r="L3" t="s">
         <v>16</v>
+      </c>
+      <c r="N3" t="str">
+        <f>N2</f>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 633</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -481,8 +502,16 @@
       <c r="B4" t="s">
         <v>15</v>
       </c>
+      <c r="C4">
+        <f t="shared" ref="C4:C9" si="1">C3</f>
+        <v>633</v>
+      </c>
       <c r="L4" t="s">
         <v>16</v>
+      </c>
+      <c r="N4" t="str">
+        <f t="shared" ref="N4:N9" si="2">N3</f>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 633</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -493,8 +522,16 @@
       <c r="B5" t="s">
         <v>15</v>
       </c>
+      <c r="C5">
+        <f t="shared" si="1"/>
+        <v>633</v>
+      </c>
       <c r="L5" t="s">
         <v>16</v>
+      </c>
+      <c r="N5" t="str">
+        <f t="shared" si="2"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 633</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -505,8 +542,16 @@
       <c r="B6" t="s">
         <v>15</v>
       </c>
+      <c r="C6">
+        <f t="shared" si="1"/>
+        <v>633</v>
+      </c>
       <c r="L6" t="s">
         <v>16</v>
+      </c>
+      <c r="N6" t="str">
+        <f t="shared" si="2"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 633</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -517,8 +562,16 @@
       <c r="B7" t="s">
         <v>15</v>
       </c>
+      <c r="C7">
+        <f t="shared" si="1"/>
+        <v>633</v>
+      </c>
       <c r="L7" t="s">
         <v>16</v>
+      </c>
+      <c r="N7" t="str">
+        <f t="shared" si="2"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 633</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -529,8 +582,16 @@
       <c r="B8" t="s">
         <v>15</v>
       </c>
+      <c r="C8">
+        <f t="shared" si="1"/>
+        <v>633</v>
+      </c>
       <c r="L8" t="s">
         <v>16</v>
+      </c>
+      <c r="N8" t="str">
+        <f t="shared" si="2"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 633</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -541,8 +602,16 @@
       <c r="B9" t="s">
         <v>15</v>
       </c>
+      <c r="C9">
+        <f t="shared" si="1"/>
+        <v>633</v>
+      </c>
       <c r="L9" t="s">
         <v>16</v>
+      </c>
+      <c r="N9" t="str">
+        <f t="shared" si="2"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 633</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -553,8 +622,14 @@
       <c r="B10" t="s">
         <v>15</v>
       </c>
+      <c r="C10">
+        <v>634</v>
+      </c>
       <c r="L10" t="s">
         <v>16</v>
+      </c>
+      <c r="N10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -565,8 +640,16 @@
       <c r="B11" t="s">
         <v>15</v>
       </c>
+      <c r="C11">
+        <f>C10</f>
+        <v>634</v>
+      </c>
       <c r="L11" t="s">
         <v>16</v>
+      </c>
+      <c r="N11" t="str">
+        <f>N10</f>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -577,8 +660,16 @@
       <c r="B12" t="s">
         <v>15</v>
       </c>
+      <c r="C12">
+        <f t="shared" ref="C12:C75" si="3">C11</f>
+        <v>634</v>
+      </c>
       <c r="L12" t="s">
         <v>16</v>
+      </c>
+      <c r="N12" t="str">
+        <f t="shared" ref="N12:N75" si="4">N11</f>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -589,8 +680,16 @@
       <c r="B13" t="s">
         <v>15</v>
       </c>
+      <c r="C13">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L13" t="s">
         <v>16</v>
+      </c>
+      <c r="N13" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -601,8 +700,16 @@
       <c r="B14" t="s">
         <v>15</v>
       </c>
+      <c r="C14">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L14" t="s">
         <v>16</v>
+      </c>
+      <c r="N14" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -613,8 +720,16 @@
       <c r="B15" t="s">
         <v>15</v>
       </c>
+      <c r="C15">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L15" t="s">
         <v>16</v>
+      </c>
+      <c r="N15" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -625,11 +740,19 @@
       <c r="B16" t="s">
         <v>15</v>
       </c>
+      <c r="C16">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L16" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:12">
+      <c r="N16" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -637,11 +760,19 @@
       <c r="B17" t="s">
         <v>15</v>
       </c>
+      <c r="C17">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L17" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:12">
+      <c r="N17" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -649,11 +780,19 @@
       <c r="B18" t="s">
         <v>15</v>
       </c>
+      <c r="C18">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:12">
+      <c r="N18" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -661,11 +800,19 @@
       <c r="B19" t="s">
         <v>15</v>
       </c>
+      <c r="C19">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L19" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="20" spans="1:12">
+      <c r="N19" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -673,11 +820,19 @@
       <c r="B20" t="s">
         <v>15</v>
       </c>
+      <c r="C20">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L20" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="21" spans="1:12">
+      <c r="N20" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -685,11 +840,19 @@
       <c r="B21" t="s">
         <v>15</v>
       </c>
+      <c r="C21">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L21" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="22" spans="1:12">
+      <c r="N21" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -697,11 +860,19 @@
       <c r="B22" t="s">
         <v>15</v>
       </c>
+      <c r="C22">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L22" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="23" spans="1:12">
+      <c r="N22" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -709,11 +880,19 @@
       <c r="B23" t="s">
         <v>15</v>
       </c>
+      <c r="C23">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L23" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="1:12">
+      <c r="N23" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -721,11 +900,19 @@
       <c r="B24" t="s">
         <v>15</v>
       </c>
+      <c r="C24">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L24" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="25" spans="1:12">
+      <c r="N24" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -733,11 +920,19 @@
       <c r="B25" t="s">
         <v>15</v>
       </c>
+      <c r="C25">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L25" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="26" spans="1:12">
+      <c r="N25" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -745,11 +940,19 @@
       <c r="B26" t="s">
         <v>15</v>
       </c>
+      <c r="C26">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L26" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="27" spans="1:12">
+      <c r="N26" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -757,11 +960,19 @@
       <c r="B27" t="s">
         <v>15</v>
       </c>
+      <c r="C27">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L27" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="28" spans="1:12">
+      <c r="N27" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -769,11 +980,19 @@
       <c r="B28" t="s">
         <v>15</v>
       </c>
+      <c r="C28">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L28" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="29" spans="1:12">
+      <c r="N28" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -781,11 +1000,19 @@
       <c r="B29" t="s">
         <v>15</v>
       </c>
+      <c r="C29">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L29" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="30" spans="1:12">
+      <c r="N29" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -793,11 +1020,19 @@
       <c r="B30" t="s">
         <v>15</v>
       </c>
+      <c r="C30">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L30" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="31" spans="1:12">
+      <c r="N30" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -805,11 +1040,19 @@
       <c r="B31" t="s">
         <v>15</v>
       </c>
+      <c r="C31">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L31" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="32" spans="1:12">
+      <c r="N31" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -817,11 +1060,19 @@
       <c r="B32" t="s">
         <v>15</v>
       </c>
+      <c r="C32">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L32" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="33" spans="1:12">
+      <c r="N32" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
       <c r="A33">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -829,11 +1080,19 @@
       <c r="B33" t="s">
         <v>15</v>
       </c>
+      <c r="C33">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L33" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="34" spans="1:12">
+      <c r="N33" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
       <c r="A34">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -841,11 +1100,19 @@
       <c r="B34" t="s">
         <v>15</v>
       </c>
+      <c r="C34">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L34" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="35" spans="1:12">
+      <c r="N34" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
       <c r="A35">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -853,11 +1120,19 @@
       <c r="B35" t="s">
         <v>15</v>
       </c>
+      <c r="C35">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L35" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="36" spans="1:12">
+      <c r="N35" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -865,11 +1140,19 @@
       <c r="B36" t="s">
         <v>15</v>
       </c>
+      <c r="C36">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L36" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="37" spans="1:12">
+      <c r="N36" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
       <c r="A37">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -877,11 +1160,19 @@
       <c r="B37" t="s">
         <v>15</v>
       </c>
+      <c r="C37">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L37" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="38" spans="1:12">
+      <c r="N37" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
       <c r="A38">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -889,11 +1180,19 @@
       <c r="B38" t="s">
         <v>15</v>
       </c>
+      <c r="C38">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L38" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="39" spans="1:12">
+      <c r="N38" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
       <c r="A39">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -901,11 +1200,19 @@
       <c r="B39" t="s">
         <v>15</v>
       </c>
+      <c r="C39">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L39" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="40" spans="1:12">
+      <c r="N39" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -913,11 +1220,19 @@
       <c r="B40" t="s">
         <v>15</v>
       </c>
+      <c r="C40">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L40" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="41" spans="1:12">
+      <c r="N40" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
       <c r="A41">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -925,11 +1240,19 @@
       <c r="B41" t="s">
         <v>15</v>
       </c>
+      <c r="C41">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L41" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="42" spans="1:12">
+      <c r="N41" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
       <c r="A42">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -937,11 +1260,19 @@
       <c r="B42" t="s">
         <v>15</v>
       </c>
+      <c r="C42">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L42" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="43" spans="1:12">
+      <c r="N42" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
       <c r="A43">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -949,11 +1280,19 @@
       <c r="B43" t="s">
         <v>15</v>
       </c>
+      <c r="C43">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L43" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="44" spans="1:12">
+      <c r="N43" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
       <c r="A44">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -961,11 +1300,19 @@
       <c r="B44" t="s">
         <v>15</v>
       </c>
+      <c r="C44">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L44" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="45" spans="1:12">
+      <c r="N44" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
       <c r="A45">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -973,11 +1320,19 @@
       <c r="B45" t="s">
         <v>15</v>
       </c>
+      <c r="C45">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L45" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="46" spans="1:12">
+      <c r="N45" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
       <c r="A46">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -985,11 +1340,19 @@
       <c r="B46" t="s">
         <v>15</v>
       </c>
+      <c r="C46">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L46" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="47" spans="1:12">
+      <c r="N46" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
       <c r="A47">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -997,11 +1360,19 @@
       <c r="B47" t="s">
         <v>15</v>
       </c>
+      <c r="C47">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L47" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="48" spans="1:12">
+      <c r="N47" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
       <c r="A48">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -1009,11 +1380,19 @@
       <c r="B48" t="s">
         <v>15</v>
       </c>
+      <c r="C48">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L48" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="49" spans="1:12">
+      <c r="N48" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14">
       <c r="A49">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -1021,11 +1400,19 @@
       <c r="B49" t="s">
         <v>15</v>
       </c>
+      <c r="C49">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L49" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="50" spans="1:12">
+      <c r="N49" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14">
       <c r="A50">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -1033,11 +1420,19 @@
       <c r="B50" t="s">
         <v>15</v>
       </c>
+      <c r="C50">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L50" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="51" spans="1:12">
+      <c r="N50" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14">
       <c r="A51">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -1045,11 +1440,19 @@
       <c r="B51" t="s">
         <v>15</v>
       </c>
+      <c r="C51">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L51" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="52" spans="1:12">
+      <c r="N51" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14">
       <c r="A52">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -1057,11 +1460,19 @@
       <c r="B52" t="s">
         <v>15</v>
       </c>
+      <c r="C52">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L52" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="53" spans="1:12">
+      <c r="N52" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14">
       <c r="A53">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -1069,11 +1480,19 @@
       <c r="B53" t="s">
         <v>15</v>
       </c>
+      <c r="C53">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L53" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="54" spans="1:12">
+      <c r="N53" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
       <c r="A54">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -1081,11 +1500,19 @@
       <c r="B54" t="s">
         <v>15</v>
       </c>
+      <c r="C54">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L54" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="55" spans="1:12">
+      <c r="N54" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14">
       <c r="A55">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -1093,11 +1520,19 @@
       <c r="B55" t="s">
         <v>15</v>
       </c>
+      <c r="C55">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L55" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="56" spans="1:12">
+      <c r="N55" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
       <c r="A56">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -1105,11 +1540,19 @@
       <c r="B56" t="s">
         <v>15</v>
       </c>
+      <c r="C56">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L56" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="57" spans="1:12">
+      <c r="N56" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14">
       <c r="A57">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -1117,11 +1560,19 @@
       <c r="B57" t="s">
         <v>15</v>
       </c>
+      <c r="C57">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L57" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="58" spans="1:12">
+      <c r="N57" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
       <c r="A58">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -1129,11 +1580,19 @@
       <c r="B58" t="s">
         <v>15</v>
       </c>
+      <c r="C58">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L58" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="59" spans="1:12">
+      <c r="N58" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14">
       <c r="A59">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -1141,11 +1600,19 @@
       <c r="B59" t="s">
         <v>15</v>
       </c>
+      <c r="C59">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L59" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="60" spans="1:12">
+      <c r="N59" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
       <c r="A60">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -1153,11 +1620,19 @@
       <c r="B60" t="s">
         <v>15</v>
       </c>
+      <c r="C60">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="61" spans="1:12">
+      <c r="N60" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14">
       <c r="A61">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -1165,11 +1640,19 @@
       <c r="B61" t="s">
         <v>15</v>
       </c>
+      <c r="C61">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L61" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="62" spans="1:12">
+      <c r="N61" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
       <c r="A62">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -1177,11 +1660,19 @@
       <c r="B62" t="s">
         <v>15</v>
       </c>
+      <c r="C62">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L62" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="63" spans="1:12">
+      <c r="N62" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14">
       <c r="A63">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -1189,11 +1680,19 @@
       <c r="B63" t="s">
         <v>15</v>
       </c>
+      <c r="C63">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L63" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="64" spans="1:12">
+      <c r="N63" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14">
       <c r="A64">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -1201,11 +1700,19 @@
       <c r="B64" t="s">
         <v>15</v>
       </c>
+      <c r="C64">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L64" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="65" spans="1:12">
+      <c r="N64" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14">
       <c r="A65">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -1213,11 +1720,19 @@
       <c r="B65" t="s">
         <v>15</v>
       </c>
+      <c r="C65">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L65" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="66" spans="1:12">
+      <c r="N65" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
       <c r="A66">
         <f t="shared" si="0"/>
         <v>65</v>
@@ -1225,11 +1740,19 @@
       <c r="B66" t="s">
         <v>15</v>
       </c>
+      <c r="C66">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L66" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="67" spans="1:12">
+      <c r="N66" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14">
       <c r="A67">
         <f t="shared" si="0"/>
         <v>66</v>
@@ -1237,764 +1760,1276 @@
       <c r="B67" t="s">
         <v>15</v>
       </c>
+      <c r="C67">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L67" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="68" spans="1:12">
+      <c r="N67" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
       <c r="A68">
-        <f t="shared" ref="A68:A130" si="1">A67+1</f>
+        <f t="shared" ref="A68:A130" si="5">A67+1</f>
         <v>67</v>
       </c>
       <c r="B68" t="s">
         <v>15</v>
       </c>
+      <c r="C68">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L68" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="69" spans="1:12">
+      <c r="N68" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
       <c r="A69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>68</v>
       </c>
       <c r="B69" t="s">
         <v>15</v>
       </c>
+      <c r="C69">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L69" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="70" spans="1:12">
+      <c r="N69" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
       <c r="A70">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>69</v>
       </c>
       <c r="B70" t="s">
         <v>15</v>
       </c>
+      <c r="C70">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L70" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="71" spans="1:12">
+      <c r="N70" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
       <c r="A71">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>70</v>
       </c>
       <c r="B71" t="s">
         <v>15</v>
       </c>
+      <c r="C71">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L71" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="72" spans="1:12">
+      <c r="N71" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
       <c r="A72">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>71</v>
       </c>
       <c r="B72" t="s">
         <v>15</v>
       </c>
+      <c r="C72">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L72" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="73" spans="1:12">
+      <c r="N72" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
       <c r="A73">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="B73" t="s">
         <v>15</v>
       </c>
+      <c r="C73">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L73" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="74" spans="1:12">
+      <c r="N73" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
       <c r="A74">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>73</v>
       </c>
       <c r="B74" t="s">
         <v>15</v>
       </c>
+      <c r="C74">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L74" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="75" spans="1:12">
+      <c r="N74" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
       <c r="A75">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>74</v>
       </c>
       <c r="B75" t="s">
         <v>15</v>
       </c>
+      <c r="C75">
+        <f t="shared" si="3"/>
+        <v>634</v>
+      </c>
       <c r="L75" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="76" spans="1:12">
+      <c r="N75" t="str">
+        <f t="shared" si="4"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
       <c r="A76">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>75</v>
       </c>
       <c r="B76" t="s">
         <v>15</v>
       </c>
+      <c r="C76">
+        <f t="shared" ref="C76:C130" si="6">C75</f>
+        <v>634</v>
+      </c>
       <c r="L76" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="77" spans="1:12">
+      <c r="N76" t="str">
+        <f t="shared" ref="N76:N130" si="7">N75</f>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
       <c r="A77">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>76</v>
       </c>
       <c r="B77" t="s">
         <v>15</v>
       </c>
+      <c r="C77">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L77" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="78" spans="1:12">
+      <c r="N77" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14">
       <c r="A78">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>77</v>
       </c>
       <c r="B78" t="s">
         <v>15</v>
       </c>
+      <c r="C78">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L78" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="79" spans="1:12">
+      <c r="N78" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14">
       <c r="A79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>78</v>
       </c>
       <c r="B79" t="s">
         <v>15</v>
       </c>
+      <c r="C79">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L79" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="80" spans="1:12">
+      <c r="N79" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14">
       <c r="A80">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>79</v>
       </c>
       <c r="B80" t="s">
         <v>15</v>
       </c>
+      <c r="C80">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L80" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="81" spans="1:12">
+      <c r="N80" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14">
       <c r="A81">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>80</v>
       </c>
       <c r="B81" t="s">
         <v>15</v>
       </c>
+      <c r="C81">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L81" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="82" spans="1:12">
+      <c r="N81" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14">
       <c r="A82">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>81</v>
       </c>
       <c r="B82" t="s">
         <v>15</v>
       </c>
+      <c r="C82">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L82" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="83" spans="1:12">
+      <c r="N82" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14">
       <c r="A83">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>82</v>
       </c>
       <c r="B83" t="s">
         <v>15</v>
       </c>
+      <c r="C83">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L83" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="84" spans="1:12">
+      <c r="N83" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14">
       <c r="A84">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>83</v>
       </c>
       <c r="B84" t="s">
         <v>15</v>
       </c>
+      <c r="C84">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L84" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="85" spans="1:12">
+      <c r="N84" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14">
       <c r="A85">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>84</v>
       </c>
       <c r="B85" t="s">
         <v>15</v>
       </c>
+      <c r="C85">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L85" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="86" spans="1:12">
+      <c r="N85" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14">
       <c r="A86">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>85</v>
       </c>
       <c r="B86" t="s">
         <v>15</v>
       </c>
+      <c r="C86">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L86" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="87" spans="1:12">
+      <c r="N86" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14">
       <c r="A87">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>86</v>
       </c>
       <c r="B87" t="s">
         <v>15</v>
       </c>
+      <c r="C87">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L87" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="88" spans="1:12">
+      <c r="N87" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14">
       <c r="A88">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>87</v>
       </c>
       <c r="B88" t="s">
         <v>15</v>
       </c>
+      <c r="C88">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L88" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="89" spans="1:12">
+      <c r="N88" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14">
       <c r="A89">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>88</v>
       </c>
       <c r="B89" t="s">
         <v>15</v>
       </c>
+      <c r="C89">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L89" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="90" spans="1:12">
+      <c r="N89" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14">
       <c r="A90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>89</v>
       </c>
       <c r="B90" t="s">
         <v>15</v>
       </c>
+      <c r="C90">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L90" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="91" spans="1:12">
+      <c r="N90" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14">
       <c r="A91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>90</v>
       </c>
       <c r="B91" t="s">
         <v>15</v>
       </c>
+      <c r="C91">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L91" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="92" spans="1:12">
+      <c r="N91" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14">
       <c r="A92">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>91</v>
       </c>
       <c r="B92" t="s">
         <v>15</v>
       </c>
+      <c r="C92">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L92" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="93" spans="1:12">
+      <c r="N92" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14">
       <c r="A93">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>92</v>
       </c>
       <c r="B93" t="s">
         <v>15</v>
       </c>
+      <c r="C93">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L93" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="94" spans="1:12">
+      <c r="N93" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14">
       <c r="A94">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>93</v>
       </c>
       <c r="B94" t="s">
         <v>15</v>
       </c>
+      <c r="C94">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L94" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="95" spans="1:12">
+      <c r="N94" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14">
       <c r="A95">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>94</v>
       </c>
       <c r="B95" t="s">
         <v>15</v>
       </c>
+      <c r="C95">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L95" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="96" spans="1:12">
+      <c r="N95" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14">
       <c r="A96">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>95</v>
       </c>
       <c r="B96" t="s">
         <v>15</v>
       </c>
+      <c r="C96">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L96" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="97" spans="1:12">
+      <c r="N96" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14">
       <c r="A97">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>96</v>
       </c>
       <c r="B97" t="s">
         <v>15</v>
       </c>
+      <c r="C97">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L97" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="98" spans="1:12">
+      <c r="N97" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14">
       <c r="A98">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>97</v>
       </c>
       <c r="B98" t="s">
         <v>15</v>
       </c>
+      <c r="C98">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L98" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="99" spans="1:12">
+      <c r="N98" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14">
       <c r="A99">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>98</v>
       </c>
       <c r="B99" t="s">
         <v>15</v>
       </c>
+      <c r="C99">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L99" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="100" spans="1:12">
+      <c r="N99" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14">
       <c r="A100">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>99</v>
       </c>
       <c r="B100" t="s">
         <v>15</v>
       </c>
+      <c r="C100">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L100" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="101" spans="1:12">
+      <c r="N100" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14">
       <c r="A101">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>100</v>
       </c>
       <c r="B101" t="s">
         <v>15</v>
       </c>
+      <c r="C101">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L101" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="102" spans="1:12">
+      <c r="N101" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14">
       <c r="A102">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>101</v>
       </c>
       <c r="B102" t="s">
         <v>15</v>
       </c>
+      <c r="C102">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L102" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="103" spans="1:12">
+      <c r="N102" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14">
       <c r="A103">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>102</v>
       </c>
       <c r="B103" t="s">
         <v>15</v>
       </c>
+      <c r="C103">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L103" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="104" spans="1:12">
+      <c r="N103" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14">
       <c r="A104">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>103</v>
       </c>
       <c r="B104" t="s">
         <v>15</v>
       </c>
+      <c r="C104">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L104" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="105" spans="1:12">
+      <c r="N104" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14">
       <c r="A105">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>104</v>
       </c>
       <c r="B105" t="s">
         <v>15</v>
       </c>
+      <c r="C105">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L105" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="106" spans="1:12">
+      <c r="N105" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14">
       <c r="A106">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>105</v>
       </c>
       <c r="B106" t="s">
         <v>15</v>
       </c>
+      <c r="C106">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L106" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="107" spans="1:12">
+      <c r="N106" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14">
       <c r="A107">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>106</v>
       </c>
       <c r="B107" t="s">
         <v>15</v>
       </c>
+      <c r="C107">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L107" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="108" spans="1:12">
+      <c r="N107" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14">
       <c r="A108">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>107</v>
       </c>
       <c r="B108" t="s">
         <v>15</v>
       </c>
+      <c r="C108">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L108" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="109" spans="1:12">
+      <c r="N108" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14">
       <c r="A109">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>108</v>
       </c>
       <c r="B109" t="s">
         <v>15</v>
       </c>
+      <c r="C109">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L109" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="110" spans="1:12">
+      <c r="N109" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14">
       <c r="A110">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>109</v>
       </c>
       <c r="B110" t="s">
         <v>15</v>
       </c>
+      <c r="C110">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L110" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="111" spans="1:12">
+      <c r="N110" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14">
       <c r="A111">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>110</v>
       </c>
       <c r="B111" t="s">
         <v>15</v>
       </c>
+      <c r="C111">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L111" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="112" spans="1:12">
+      <c r="N111" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14">
       <c r="A112">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>111</v>
       </c>
       <c r="B112" t="s">
         <v>15</v>
       </c>
+      <c r="C112">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L112" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="113" spans="1:12">
+      <c r="N112" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14">
       <c r="A113">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>112</v>
       </c>
       <c r="B113" t="s">
         <v>15</v>
       </c>
+      <c r="C113">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L113" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="114" spans="1:12">
+      <c r="N113" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14">
       <c r="A114">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>113</v>
       </c>
       <c r="B114" t="s">
         <v>15</v>
       </c>
+      <c r="C114">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L114" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="115" spans="1:12">
+      <c r="N114" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14">
       <c r="A115">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>114</v>
       </c>
       <c r="B115" t="s">
         <v>15</v>
       </c>
+      <c r="C115">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L115" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="116" spans="1:12">
+      <c r="N115" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14">
       <c r="A116">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>115</v>
       </c>
       <c r="B116" t="s">
         <v>15</v>
       </c>
+      <c r="C116">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L116" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="117" spans="1:12">
+      <c r="N116" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14">
       <c r="A117">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>116</v>
       </c>
       <c r="B117" t="s">
         <v>15</v>
       </c>
+      <c r="C117">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L117" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="118" spans="1:12">
+      <c r="N117" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14">
       <c r="A118">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>117</v>
       </c>
       <c r="B118" t="s">
         <v>15</v>
       </c>
+      <c r="C118">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L118" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="119" spans="1:12">
+      <c r="N118" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14">
       <c r="A119">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>118</v>
       </c>
       <c r="B119" t="s">
         <v>15</v>
       </c>
+      <c r="C119">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L119" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="120" spans="1:12">
+      <c r="N119" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14">
       <c r="A120">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>119</v>
       </c>
       <c r="B120" t="s">
         <v>15</v>
       </c>
+      <c r="C120">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L120" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="121" spans="1:12">
+      <c r="N120" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14">
       <c r="A121">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>120</v>
       </c>
       <c r="B121" t="s">
         <v>15</v>
       </c>
+      <c r="C121">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L121" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="122" spans="1:12">
+      <c r="N121" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14">
       <c r="A122">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>121</v>
       </c>
       <c r="B122" t="s">
         <v>15</v>
       </c>
+      <c r="C122">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L122" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="123" spans="1:12">
+      <c r="N122" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="123" spans="1:14">
       <c r="A123">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>122</v>
       </c>
       <c r="B123" t="s">
         <v>15</v>
       </c>
+      <c r="C123">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L123" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="124" spans="1:12">
+      <c r="N123" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14">
       <c r="A124">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>123</v>
       </c>
       <c r="B124" t="s">
         <v>15</v>
       </c>
+      <c r="C124">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L124" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="125" spans="1:12">
+      <c r="N124" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="125" spans="1:14">
       <c r="A125">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>124</v>
       </c>
       <c r="B125" t="s">
         <v>15</v>
       </c>
+      <c r="C125">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L125" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="126" spans="1:12">
+      <c r="N125" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="126" spans="1:14">
       <c r="A126">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>125</v>
       </c>
       <c r="B126" t="s">
         <v>15</v>
       </c>
+      <c r="C126">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L126" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="127" spans="1:12">
+      <c r="N126" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="127" spans="1:14">
       <c r="A127">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>126</v>
       </c>
       <c r="B127" t="s">
         <v>15</v>
       </c>
+      <c r="C127">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L127" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="128" spans="1:12">
+      <c r="N127" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="128" spans="1:14">
       <c r="A128">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>127</v>
       </c>
       <c r="B128" t="s">
         <v>15</v>
       </c>
+      <c r="C128">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L128" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="129" spans="1:12">
+      <c r="N128" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="129" spans="1:14">
       <c r="A129">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>128</v>
       </c>
       <c r="B129" t="s">
         <v>15</v>
       </c>
+      <c r="C129">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L129" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="130" spans="1:12">
+      <c r="N129" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
+      </c>
+    </row>
+    <row r="130" spans="1:14">
       <c r="A130">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>129</v>
       </c>
       <c r="B130" t="s">
         <v>15</v>
       </c>
+      <c r="C130">
+        <f t="shared" si="6"/>
+        <v>634</v>
+      </c>
       <c r="L130" t="s">
         <v>16</v>
+      </c>
+      <c r="N130" t="str">
+        <f t="shared" si="7"/>
+        <v>Dawes Rolls Full Document - Creek By Blood - Page 634</v>
       </c>
     </row>
   </sheetData>

</xml_diff>